<commit_message>
Update E2E test cases, security reports, and workflows for GitHub Actions
</commit_message>
<xml_diff>
--- a/SmartLearn_LoadTest_Report.xlsx
+++ b/SmartLearn_LoadTest_Report.xlsx
@@ -936,7 +936,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run Date: 9/7/2026, 2:14:49 pm  |  Target Endpoint: http://localhost:8080/api/auth/user  |  Duration: 60s</t>
+          <t>Run Date: 22/7/2026, 10:38:38 am  |  Target Endpoint: http://localhost:8080/api/auth/user  |  Duration: 60s</t>
         </is>
       </c>
     </row>
@@ -945,7 +945,7 @@
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>TOTAL REQUESTS
-424105</t>
+210773</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -957,19 +957,19 @@
       <c r="E4" s="5" t="inlineStr">
         <is>
           <t>AVG LATENCY
-14.2ms</t>
+28.5ms</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
           <t>THROUGHPUT
-7061.7 RPS</t>
+3508.9 RPS</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
           <t>99th PERCENTILE
-25ms</t>
+243ms</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="I9" s="11" t="inlineStr">
         <is>
-          <t>7 ms</t>
+          <t>8 ms</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
-          <t>13 ms</t>
+          <t>17 ms</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
-          <t>18 ms</t>
+          <t>27 ms</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>60.06 seconds</t>
+          <t>60.07 seconds</t>
         </is>
       </c>
       <c r="F12" s="12" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="I12" s="16" t="inlineStr">
         <is>
-          <t>21 ms</t>
+          <t>147 ms</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>9/7/2026, 2:14:49 pm</t>
+          <t>22/7/2026, 10:38:38 am</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="I13" s="17" t="inlineStr">
         <is>
-          <t>25 ms</t>
+          <t>243 ms</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>9/7/2026, 2:15:49 pm</t>
+          <t>22/7/2026, 10:39:38 am</t>
         </is>
       </c>
       <c r="F14" s="12" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="I14" s="18" t="inlineStr">
         <is>
-          <t>91 ms</t>
+          <t>807 ms</t>
         </is>
       </c>
     </row>
@@ -1125,9 +1125,9 @@
       <c r="A16" s="19" t="inlineStr">
         <is>
           <t>📖 BASELINE TEST INTERPRETATION GUIDELINE:
-• Requests per Second (RPS): This tells you the capacity the server handles concurrently. Under 100 concurrent virtual users, your API successfully handled an average of 7061.71 requests/sec.
-• Response Time: Response times below 200ms are considered excellent. Your median response time (p50) was 13ms, and the overall average was 14.15ms.
-• High Percentiles (p90, p99): p99 indicates the latency for the slowest 1% of users. Here, 99% of requests completed under 25ms, proving excellent stability under expected concurrency.</t>
+• Requests per Second (RPS): This tells you the capacity the server handles concurrently. Under 100 concurrent virtual users, your API successfully handled an average of 3508.91 requests/sec.
+• Response Time: Response times below 200ms are considered excellent. Your median response time (p50) was 17ms, and the overall average was 28.47ms.
+• High Percentiles (p90, p99): p99 indicates the latency for the slowest 1% of users. Here, 99% of requests completed under 243ms, proving excellent stability under expected concurrency.</t>
         </is>
       </c>
     </row>
@@ -1233,16 +1233,16 @@
         </is>
       </c>
       <c r="B3" s="23" t="n">
-        <v>4581</v>
+        <v>3610</v>
       </c>
       <c r="C3" s="24" t="n">
-        <v>4581</v>
+        <v>3610</v>
       </c>
       <c r="D3" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E3" s="25" t="n">
-        <v>21.1</v>
+        <v>26.7</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
@@ -1252,16 +1252,16 @@
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>6185</v>
+        <v>4749</v>
       </c>
       <c r="C4" s="28" t="n">
-        <v>6185</v>
+        <v>4749</v>
       </c>
       <c r="D4" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>16.1</v>
+        <v>21.1</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -1271,16 +1271,16 @@
         </is>
       </c>
       <c r="B5" s="23" t="n">
-        <v>6853</v>
+        <v>4954</v>
       </c>
       <c r="C5" s="24" t="n">
-        <v>6853</v>
+        <v>4954</v>
       </c>
       <c r="D5" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="25" t="n">
-        <v>14.6</v>
+        <v>20.1</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
@@ -1290,16 +1290,16 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>6882</v>
+        <v>5873</v>
       </c>
       <c r="C6" s="28" t="n">
-        <v>6882</v>
+        <v>5873</v>
       </c>
       <c r="D6" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>14.5</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
@@ -1309,16 +1309,16 @@
         </is>
       </c>
       <c r="B7" s="23" t="n">
-        <v>6967</v>
+        <v>4759</v>
       </c>
       <c r="C7" s="24" t="n">
-        <v>6967</v>
+        <v>4759</v>
       </c>
       <c r="D7" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="25" t="n">
-        <v>14.4</v>
+        <v>21.2</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -1328,16 +1328,16 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>7009</v>
+        <v>5086</v>
       </c>
       <c r="C8" s="28" t="n">
-        <v>7009</v>
+        <v>5086</v>
       </c>
       <c r="D8" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>14.3</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -1347,16 +1347,16 @@
         </is>
       </c>
       <c r="B9" s="23" t="n">
-        <v>6916</v>
+        <v>5269</v>
       </c>
       <c r="C9" s="24" t="n">
-        <v>6916</v>
+        <v>5269</v>
       </c>
       <c r="D9" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="25" t="n">
-        <v>14.4</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -1366,16 +1366,16 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>7101</v>
+        <v>5637</v>
       </c>
       <c r="C10" s="28" t="n">
-        <v>7101</v>
+        <v>5637</v>
       </c>
       <c r="D10" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>14.1</v>
+        <v>17.7</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
@@ -1385,16 +1385,16 @@
         </is>
       </c>
       <c r="B11" s="23" t="n">
-        <v>6996</v>
+        <v>6110</v>
       </c>
       <c r="C11" s="24" t="n">
-        <v>6996</v>
+        <v>6110</v>
       </c>
       <c r="D11" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="25" t="n">
-        <v>14.3</v>
+        <v>16.4</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
@@ -1404,16 +1404,16 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>6936</v>
+        <v>6177</v>
       </c>
       <c r="C12" s="28" t="n">
-        <v>6936</v>
+        <v>6177</v>
       </c>
       <c r="D12" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>14.4</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
@@ -1423,16 +1423,16 @@
         </is>
       </c>
       <c r="B13" s="23" t="n">
-        <v>6945</v>
+        <v>6359</v>
       </c>
       <c r="C13" s="24" t="n">
-        <v>6945</v>
+        <v>6359</v>
       </c>
       <c r="D13" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="25" t="n">
-        <v>14.4</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
@@ -1442,16 +1442,16 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>6939</v>
+        <v>6129</v>
       </c>
       <c r="C14" s="28" t="n">
-        <v>6939</v>
+        <v>6129</v>
       </c>
       <c r="D14" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>14.4</v>
+        <v>16.3</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -1461,16 +1461,16 @@
         </is>
       </c>
       <c r="B15" s="23" t="n">
-        <v>7112</v>
+        <v>6134</v>
       </c>
       <c r="C15" s="24" t="n">
-        <v>7112</v>
+        <v>6134</v>
       </c>
       <c r="D15" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="25" t="n">
-        <v>14.1</v>
+        <v>16.3</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
@@ -1480,16 +1480,16 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>6844</v>
+        <v>6204</v>
       </c>
       <c r="C16" s="28" t="n">
-        <v>6844</v>
+        <v>6204</v>
       </c>
       <c r="D16" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>14.7</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
@@ -1499,16 +1499,16 @@
         </is>
       </c>
       <c r="B17" s="23" t="n">
-        <v>7035</v>
+        <v>6263</v>
       </c>
       <c r="C17" s="24" t="n">
-        <v>7035</v>
+        <v>6263</v>
       </c>
       <c r="D17" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E17" s="25" t="n">
-        <v>14.1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
@@ -1518,16 +1518,16 @@
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>7053</v>
+        <v>5983</v>
       </c>
       <c r="C18" s="28" t="n">
-        <v>7053</v>
+        <v>5983</v>
       </c>
       <c r="D18" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>14.2</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
@@ -1537,16 +1537,16 @@
         </is>
       </c>
       <c r="B19" s="23" t="n">
-        <v>7089</v>
+        <v>6345</v>
       </c>
       <c r="C19" s="24" t="n">
-        <v>7089</v>
+        <v>6345</v>
       </c>
       <c r="D19" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E19" s="25" t="n">
-        <v>14.1</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -1556,16 +1556,16 @@
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>7198</v>
+        <v>6282</v>
       </c>
       <c r="C20" s="28" t="n">
-        <v>7198</v>
+        <v>6282</v>
       </c>
       <c r="D20" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>13.9</v>
+        <v>15.9</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
@@ -1575,16 +1575,16 @@
         </is>
       </c>
       <c r="B21" s="23" t="n">
-        <v>6651</v>
+        <v>6349</v>
       </c>
       <c r="C21" s="24" t="n">
-        <v>6651</v>
+        <v>6349</v>
       </c>
       <c r="D21" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="25" t="n">
-        <v>15.1</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
@@ -1594,16 +1594,16 @@
         </is>
       </c>
       <c r="B22" s="27" t="n">
-        <v>7281</v>
+        <v>5649</v>
       </c>
       <c r="C22" s="28" t="n">
-        <v>7281</v>
+        <v>5649</v>
       </c>
       <c r="D22" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="29" t="n">
-        <v>13.8</v>
+        <v>17.7</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
@@ -1613,16 +1613,16 @@
         </is>
       </c>
       <c r="B23" s="23" t="n">
-        <v>7175</v>
+        <v>4970</v>
       </c>
       <c r="C23" s="24" t="n">
-        <v>7175</v>
+        <v>4970</v>
       </c>
       <c r="D23" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E23" s="25" t="n">
-        <v>13.9</v>
+        <v>21.2</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
@@ -1632,16 +1632,16 @@
         </is>
       </c>
       <c r="B24" s="27" t="n">
-        <v>7162</v>
+        <v>642</v>
       </c>
       <c r="C24" s="28" t="n">
-        <v>7162</v>
+        <v>642</v>
       </c>
       <c r="D24" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="29" t="n">
-        <v>13.9</v>
+        <v>158.1</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
@@ -1651,16 +1651,16 @@
         </is>
       </c>
       <c r="B25" s="23" t="n">
-        <v>6993</v>
+        <v>624</v>
       </c>
       <c r="C25" s="24" t="n">
-        <v>6993</v>
+        <v>624</v>
       </c>
       <c r="D25" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="25" t="n">
-        <v>14.3</v>
+        <v>166.6</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
@@ -1670,16 +1670,16 @@
         </is>
       </c>
       <c r="B26" s="27" t="n">
-        <v>7006</v>
+        <v>417</v>
       </c>
       <c r="C26" s="28" t="n">
-        <v>7006</v>
+        <v>417</v>
       </c>
       <c r="D26" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E26" s="29" t="n">
-        <v>14.3</v>
+        <v>245.9</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
@@ -1689,16 +1689,16 @@
         </is>
       </c>
       <c r="B27" s="23" t="n">
-        <v>7254</v>
+        <v>237</v>
       </c>
       <c r="C27" s="24" t="n">
-        <v>7254</v>
+        <v>237</v>
       </c>
       <c r="D27" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E27" s="25" t="n">
-        <v>13.8</v>
+        <v>413.9</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
@@ -1708,16 +1708,16 @@
         </is>
       </c>
       <c r="B28" s="27" t="n">
-        <v>7159</v>
+        <v>462</v>
       </c>
       <c r="C28" s="28" t="n">
-        <v>7159</v>
+        <v>462</v>
       </c>
       <c r="D28" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E28" s="29" t="n">
-        <v>13.9</v>
+        <v>209</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
@@ -1727,16 +1727,16 @@
         </is>
       </c>
       <c r="B29" s="23" t="n">
-        <v>7307</v>
+        <v>468</v>
       </c>
       <c r="C29" s="24" t="n">
-        <v>7307</v>
+        <v>468</v>
       </c>
       <c r="D29" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E29" s="25" t="n">
-        <v>13.7</v>
+        <v>215.3</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
@@ -1746,16 +1746,16 @@
         </is>
       </c>
       <c r="B30" s="27" t="n">
-        <v>7161</v>
+        <v>418</v>
       </c>
       <c r="C30" s="28" t="n">
-        <v>7161</v>
+        <v>418</v>
       </c>
       <c r="D30" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E30" s="29" t="n">
-        <v>13.9</v>
+        <v>244.3</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
@@ -1765,16 +1765,16 @@
         </is>
       </c>
       <c r="B31" s="23" t="n">
-        <v>7188</v>
+        <v>588</v>
       </c>
       <c r="C31" s="24" t="n">
-        <v>7188</v>
+        <v>588</v>
       </c>
       <c r="D31" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E31" s="25" t="n">
-        <v>13.9</v>
+        <v>159.1</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
@@ -1784,16 +1784,16 @@
         </is>
       </c>
       <c r="B32" s="27" t="n">
-        <v>7082</v>
+        <v>678</v>
       </c>
       <c r="C32" s="28" t="n">
-        <v>7082</v>
+        <v>678</v>
       </c>
       <c r="D32" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E32" s="29" t="n">
-        <v>14.1</v>
+        <v>168.7</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
@@ -1803,16 +1803,16 @@
         </is>
       </c>
       <c r="B33" s="23" t="n">
-        <v>7243</v>
+        <v>633</v>
       </c>
       <c r="C33" s="24" t="n">
-        <v>7243</v>
+        <v>633</v>
       </c>
       <c r="D33" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E33" s="25" t="n">
-        <v>13.8</v>
+        <v>135.2</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
@@ -1822,16 +1822,16 @@
         </is>
       </c>
       <c r="B34" s="27" t="n">
-        <v>7267</v>
+        <v>640</v>
       </c>
       <c r="C34" s="28" t="n">
-        <v>7267</v>
+        <v>640</v>
       </c>
       <c r="D34" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E34" s="29" t="n">
-        <v>13.8</v>
+        <v>165.2</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
@@ -1841,16 +1841,16 @@
         </is>
       </c>
       <c r="B35" s="23" t="n">
-        <v>7149</v>
+        <v>470</v>
       </c>
       <c r="C35" s="24" t="n">
-        <v>7149</v>
+        <v>470</v>
       </c>
       <c r="D35" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E35" s="25" t="n">
-        <v>13.9</v>
+        <v>217.3</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
@@ -1860,16 +1860,16 @@
         </is>
       </c>
       <c r="B36" s="27" t="n">
-        <v>7149</v>
+        <v>466</v>
       </c>
       <c r="C36" s="28" t="n">
-        <v>7149</v>
+        <v>466</v>
       </c>
       <c r="D36" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E36" s="29" t="n">
-        <v>14</v>
+        <v>208.5</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
@@ -1879,16 +1879,16 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>7125</v>
+        <v>461</v>
       </c>
       <c r="C37" s="24" t="n">
-        <v>7125</v>
+        <v>461</v>
       </c>
       <c r="D37" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E37" s="25" t="n">
-        <v>14</v>
+        <v>219.6</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
@@ -1898,16 +1898,16 @@
         </is>
       </c>
       <c r="B38" s="27" t="n">
-        <v>7273</v>
+        <v>455</v>
       </c>
       <c r="C38" s="28" t="n">
-        <v>7273</v>
+        <v>455</v>
       </c>
       <c r="D38" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E38" s="29" t="n">
-        <v>13.8</v>
+        <v>221.4</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
@@ -1917,16 +1917,16 @@
         </is>
       </c>
       <c r="B39" s="23" t="n">
-        <v>7132</v>
+        <v>404</v>
       </c>
       <c r="C39" s="24" t="n">
-        <v>7132</v>
+        <v>404</v>
       </c>
       <c r="D39" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E39" s="25" t="n">
-        <v>14</v>
+        <v>247.6</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
@@ -1936,16 +1936,16 @@
         </is>
       </c>
       <c r="B40" s="27" t="n">
-        <v>7209</v>
+        <v>388</v>
       </c>
       <c r="C40" s="28" t="n">
-        <v>7209</v>
+        <v>388</v>
       </c>
       <c r="D40" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E40" s="29" t="n">
-        <v>13.9</v>
+        <v>248.6</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
@@ -1955,16 +1955,16 @@
         </is>
       </c>
       <c r="B41" s="23" t="n">
-        <v>6696</v>
+        <v>503</v>
       </c>
       <c r="C41" s="24" t="n">
-        <v>6696</v>
+        <v>503</v>
       </c>
       <c r="D41" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E41" s="25" t="n">
-        <v>14.9</v>
+        <v>201.1</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
@@ -1974,16 +1974,16 @@
         </is>
       </c>
       <c r="B42" s="27" t="n">
-        <v>7284</v>
+        <v>474</v>
       </c>
       <c r="C42" s="28" t="n">
-        <v>7284</v>
+        <v>474</v>
       </c>
       <c r="D42" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E42" s="29" t="n">
-        <v>13.7</v>
+        <v>208.4</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
@@ -1993,16 +1993,16 @@
         </is>
       </c>
       <c r="B43" s="23" t="n">
-        <v>7105</v>
+        <v>628</v>
       </c>
       <c r="C43" s="24" t="n">
-        <v>7105</v>
+        <v>628</v>
       </c>
       <c r="D43" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E43" s="25" t="n">
-        <v>14.1</v>
+        <v>157.5</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
@@ -2012,16 +2012,16 @@
         </is>
       </c>
       <c r="B44" s="27" t="n">
-        <v>7131</v>
+        <v>541</v>
       </c>
       <c r="C44" s="28" t="n">
-        <v>7131</v>
+        <v>541</v>
       </c>
       <c r="D44" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E44" s="29" t="n">
-        <v>14</v>
+        <v>185.9</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
@@ -2031,16 +2031,16 @@
         </is>
       </c>
       <c r="B45" s="23" t="n">
-        <v>7245</v>
+        <v>579</v>
       </c>
       <c r="C45" s="24" t="n">
-        <v>7245</v>
+        <v>579</v>
       </c>
       <c r="D45" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E45" s="25" t="n">
-        <v>13.8</v>
+        <v>172.8</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
@@ -2050,16 +2050,16 @@
         </is>
       </c>
       <c r="B46" s="27" t="n">
-        <v>7195</v>
+        <v>556</v>
       </c>
       <c r="C46" s="28" t="n">
-        <v>7195</v>
+        <v>556</v>
       </c>
       <c r="D46" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E46" s="29" t="n">
-        <v>14</v>
+        <v>177.5</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
@@ -2069,16 +2069,16 @@
         </is>
       </c>
       <c r="B47" s="23" t="n">
-        <v>7225</v>
+        <v>541</v>
       </c>
       <c r="C47" s="24" t="n">
-        <v>7225</v>
+        <v>541</v>
       </c>
       <c r="D47" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E47" s="25" t="n">
-        <v>13.8</v>
+        <v>202.4</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
@@ -2088,16 +2088,16 @@
         </is>
       </c>
       <c r="B48" s="27" t="n">
-        <v>7296</v>
+        <v>426</v>
       </c>
       <c r="C48" s="28" t="n">
-        <v>7296</v>
+        <v>426</v>
       </c>
       <c r="D48" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E48" s="29" t="n">
-        <v>13.7</v>
+        <v>213.6</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
@@ -2107,16 +2107,16 @@
         </is>
       </c>
       <c r="B49" s="23" t="n">
-        <v>7162</v>
+        <v>4467</v>
       </c>
       <c r="C49" s="24" t="n">
-        <v>7162</v>
+        <v>4467</v>
       </c>
       <c r="D49" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E49" s="25" t="n">
-        <v>14</v>
+        <v>20.7</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
@@ -2126,16 +2126,16 @@
         </is>
       </c>
       <c r="B50" s="27" t="n">
-        <v>7173</v>
+        <v>5981</v>
       </c>
       <c r="C50" s="28" t="n">
-        <v>7173</v>
+        <v>5981</v>
       </c>
       <c r="D50" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E50" s="29" t="n">
-        <v>13.9</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
@@ -2145,16 +2145,16 @@
         </is>
       </c>
       <c r="B51" s="23" t="n">
-        <v>7254</v>
+        <v>5939</v>
       </c>
       <c r="C51" s="24" t="n">
-        <v>7254</v>
+        <v>5939</v>
       </c>
       <c r="D51" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E51" s="25" t="n">
-        <v>13.8</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -2164,16 +2164,16 @@
         </is>
       </c>
       <c r="B52" s="27" t="n">
-        <v>7183</v>
+        <v>6042</v>
       </c>
       <c r="C52" s="28" t="n">
-        <v>7183</v>
+        <v>6042</v>
       </c>
       <c r="D52" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E52" s="29" t="n">
-        <v>13.9</v>
+        <v>16.6</v>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
@@ -2183,16 +2183,16 @@
         </is>
       </c>
       <c r="B53" s="23" t="n">
-        <v>7291</v>
+        <v>6248</v>
       </c>
       <c r="C53" s="24" t="n">
-        <v>7291</v>
+        <v>6248</v>
       </c>
       <c r="D53" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E53" s="25" t="n">
-        <v>13.7</v>
+        <v>15.9</v>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
@@ -2202,16 +2202,16 @@
         </is>
       </c>
       <c r="B54" s="27" t="n">
-        <v>7095</v>
+        <v>6034</v>
       </c>
       <c r="C54" s="28" t="n">
-        <v>7095</v>
+        <v>6034</v>
       </c>
       <c r="D54" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E54" s="29" t="n">
-        <v>14.1</v>
+        <v>16.6</v>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
@@ -2221,16 +2221,16 @@
         </is>
       </c>
       <c r="B55" s="23" t="n">
-        <v>7192</v>
+        <v>6166</v>
       </c>
       <c r="C55" s="24" t="n">
-        <v>7192</v>
+        <v>6166</v>
       </c>
       <c r="D55" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E55" s="25" t="n">
-        <v>13.9</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
@@ -2240,16 +2240,16 @@
         </is>
       </c>
       <c r="B56" s="27" t="n">
-        <v>7276</v>
+        <v>5142</v>
       </c>
       <c r="C56" s="28" t="n">
-        <v>7276</v>
+        <v>5142</v>
       </c>
       <c r="D56" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E56" s="29" t="n">
-        <v>13.7</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
@@ -2259,16 +2259,16 @@
         </is>
       </c>
       <c r="B57" s="23" t="n">
-        <v>7185</v>
+        <v>5316</v>
       </c>
       <c r="C57" s="24" t="n">
-        <v>7185</v>
+        <v>5316</v>
       </c>
       <c r="D57" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E57" s="25" t="n">
-        <v>13.9</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
@@ -2278,16 +2278,16 @@
         </is>
       </c>
       <c r="B58" s="27" t="n">
-        <v>7308</v>
+        <v>5069</v>
       </c>
       <c r="C58" s="28" t="n">
-        <v>7308</v>
+        <v>5069</v>
       </c>
       <c r="D58" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E58" s="29" t="n">
-        <v>13.7</v>
+        <v>19.7</v>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
@@ -2297,16 +2297,16 @@
         </is>
       </c>
       <c r="B59" s="23" t="n">
-        <v>7183</v>
+        <v>5204</v>
       </c>
       <c r="C59" s="24" t="n">
-        <v>7183</v>
+        <v>5204</v>
       </c>
       <c r="D59" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E59" s="25" t="n">
-        <v>13.9</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
@@ -2316,16 +2316,16 @@
         </is>
       </c>
       <c r="B60" s="27" t="n">
-        <v>7232</v>
+        <v>5516</v>
       </c>
       <c r="C60" s="28" t="n">
-        <v>7232</v>
+        <v>5516</v>
       </c>
       <c r="D60" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E60" s="29" t="n">
-        <v>13.9</v>
+        <v>18.2</v>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
@@ -2335,16 +2335,16 @@
         </is>
       </c>
       <c r="B61" s="23" t="n">
-        <v>7209</v>
+        <v>5840</v>
       </c>
       <c r="C61" s="24" t="n">
-        <v>7209</v>
+        <v>5840</v>
       </c>
       <c r="D61" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E61" s="25" t="n">
-        <v>13.8</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
@@ -2354,16 +2354,16 @@
         </is>
       </c>
       <c r="B62" s="27" t="n">
-        <v>7264</v>
+        <v>5921</v>
       </c>
       <c r="C62" s="28" t="n">
-        <v>7264</v>
+        <v>5921</v>
       </c>
       <c r="D62" s="28" t="n">
         <v>0</v>
       </c>
       <c r="E62" s="29" t="n">
-        <v>13.8</v>
+        <v>16.9</v>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
@@ -2373,16 +2373,16 @@
         </is>
       </c>
       <c r="B63" s="23" t="n">
-        <v>314</v>
+        <v>298</v>
       </c>
       <c r="C63" s="24" t="n">
-        <v>314</v>
+        <v>298</v>
       </c>
       <c r="D63" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E63" s="25" t="n">
-        <v>15.1</v>
+        <v>18.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>